<commit_message>
Vault sync: Nobunaga emulator toolchain reorg + econ/combat findings
- Reorganize nobunaga scripts under tools/ (VM emulator, renderers, decoders)
- Add disasm VM dumps, command docs, atlas renders, appendix formulas
- Update mesen-labels, vm-opcodes, shared game-annotation tools
- Gitignore multi-hundred-MB regenerable emulator trace dumps (keep .dmp snapshots)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/game-annotation/nobunaga/17fief.xlsx
+++ b/projects/game-annotation/nobunaga/17fief.xlsx
@@ -8,19 +8,38 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris.Isaacson\Vault\projects\game-annotation\nobunaga\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7176BF6-4A4A-4741-AADD-E2805A783833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1BCCF03-F6CD-4608-B6D9-909CE8A2401A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5730" yWindow="3165" windowWidth="21600" windowHeight="12645" xr2:uid="{FDB40808-8C5F-486C-AF63-A8D18F3A0A01}"/>
+    <workbookView xWindow="28680" yWindow="-255" windowWidth="29040" windowHeight="17520" xr2:uid="{FDB40808-8C5F-486C-AF63-A8D18F3A0A01}"/>
   </bookViews>
   <sheets>
     <sheet name="17fief" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'17fief'!$A$1:$AN$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Sheet1!$A$2:$B$13</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="130">
   <si>
     <t>idx</t>
   </si>
@@ -278,6 +297,138 @@
   </si>
   <si>
     <t>7,8,12</t>
+  </si>
+  <si>
+    <t>Rk</t>
+  </si>
+  <si>
+    <t>Adj</t>
+  </si>
+  <si>
+    <t>AJP</t>
+  </si>
+  <si>
+    <t>2,16,7</t>
+  </si>
+  <si>
+    <t>10,16,5,1</t>
+  </si>
+  <si>
+    <t>AvAdP</t>
+  </si>
+  <si>
+    <t>4,10,5</t>
+  </si>
+  <si>
+    <t>3,13,5</t>
+  </si>
+  <si>
+    <t>4,3,13,12,10,2,16</t>
+  </si>
+  <si>
+    <t>15,11</t>
+  </si>
+  <si>
+    <t>16,15,8,17,1</t>
+  </si>
+  <si>
+    <t>9,16,17,7,11</t>
+  </si>
+  <si>
+    <t>13,12,16,8</t>
+  </si>
+  <si>
+    <t>3,2,5</t>
+  </si>
+  <si>
+    <t>15,8,17,6</t>
+  </si>
+  <si>
+    <t>13,9,16,5</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>14,4,9,12,5</t>
+  </si>
+  <si>
+    <t>17,7,11,6</t>
+  </si>
+  <si>
+    <t>9,12,2,8,7,5,1</t>
+  </si>
+  <si>
+    <t>15,8,7,11</t>
+  </si>
+  <si>
+    <t>AvAdjA</t>
+  </si>
+  <si>
+    <t>AdjA</t>
+  </si>
+  <si>
+    <t>AdjR</t>
+  </si>
+  <si>
+    <t>AdjAR</t>
+  </si>
+  <si>
+    <t>3,14,2</t>
+  </si>
+  <si>
+    <t>14,16,9,17,1</t>
+  </si>
+  <si>
+    <t>4,14,5,1</t>
+  </si>
+  <si>
+    <t>7,3,5</t>
+  </si>
+  <si>
+    <t>6,7,15,11,4,3,14</t>
+  </si>
+  <si>
+    <t>7,15,5</t>
+  </si>
+  <si>
+    <t>6,4,5</t>
+  </si>
+  <si>
+    <t>16,12</t>
+  </si>
+  <si>
+    <t>10,14,17,2,12</t>
+  </si>
+  <si>
+    <t>15,11,14,9</t>
+  </si>
+  <si>
+    <t>15,10,14,5</t>
+  </si>
+  <si>
+    <t>16,9,17,8</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>10,11,3,9,2,5,1</t>
+  </si>
+  <si>
+    <t>13,6,10,11,5</t>
+  </si>
+  <si>
+    <t>17,2,12,8</t>
+  </si>
+  <si>
+    <t>16,9,2,12</t>
+  </si>
+  <si>
+    <t>xsRice</t>
+  </si>
+  <si>
+    <t>riottax</t>
   </si>
 </sst>
 </file>
@@ -433,7 +584,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -613,6 +764,18 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -774,11 +937,15 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1154,7 +1321,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94A9DEAF-4754-41E1-A6D8-10B03E1EEF36}">
-  <dimension ref="A1:AF18"/>
+  <dimension ref="A1:AS27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.5703125" bestFit="1" customWidth="1"/>
@@ -1188,9 +1355,16 @@
     <col min="30" max="30" width="6.28515625" customWidth="1"/>
     <col min="31" max="31" width="4.42578125" customWidth="1"/>
     <col min="32" max="32" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="12.28515625" hidden="1" customWidth="1"/>
+    <col min="34" max="34" width="5.85546875" hidden="1" customWidth="1"/>
+    <col min="35" max="35" width="7.140625" customWidth="1"/>
+    <col min="36" max="36" width="11.28515625" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="7" hidden="1" customWidth="1"/>
+    <col min="38" max="38" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="4.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1281,110 +1455,172 @@
       <c r="AD1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AE1" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>87</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>88</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>91</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>109</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>108</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>107</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>110</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>128</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>16</v>
-      </c>
-      <c r="B2" t="s">
-        <v>31</v>
       </c>
       <c r="C2">
         <v>1000</v>
       </c>
       <c r="D2">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="G2">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H2">
         <v>80</v>
       </c>
       <c r="I2">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="J2">
+        <v>79</v>
+      </c>
+      <c r="K2">
+        <v>70</v>
+      </c>
+      <c r="L2">
+        <v>74</v>
+      </c>
+      <c r="M2">
+        <v>74</v>
+      </c>
+      <c r="N2">
+        <v>61</v>
+      </c>
+      <c r="O2">
         <v>71</v>
       </c>
-      <c r="K2">
-        <v>72</v>
-      </c>
-      <c r="L2">
-        <v>78</v>
-      </c>
-      <c r="M2">
-        <v>77</v>
-      </c>
-      <c r="N2">
-        <v>78</v>
-      </c>
-      <c r="O2">
-        <v>80</v>
-      </c>
       <c r="P2">
-        <f>(L2*N2*O2)^(1/3)</f>
-        <v>78.661048467230643</v>
+        <f t="shared" ref="P2:P18" si="0">(L2*N2*O2)^(1/3)</f>
+        <v>68.434216775695589</v>
       </c>
       <c r="Q2">
-        <f>(F2*H2*K2)^(1/3)</f>
-        <v>69.38785980258659</v>
+        <f t="shared" ref="Q2:Q18" si="1">(F2*H2*K2)^(1/3)</f>
+        <v>64.537145840981722</v>
       </c>
       <c r="R2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="S2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="T2">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="U2">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="V2">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="W2">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="X2">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="Y2">
         <v>0</v>
       </c>
       <c r="Z2">
-        <f>(T2*U2*V2*W2*X2)^(1/5)</f>
-        <v>108.3103906739629</v>
+        <f t="shared" ref="Z2:Z18" si="2">(T2*U2*V2*W2*X2)^(1/5)</f>
+        <v>99.219302709069495</v>
       </c>
       <c r="AA2" s="2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AB2" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AC2" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AD2">
-        <f>(P2*Q2*Z2)^(1/3)</f>
-        <v>83.92753126291089</v>
+        <f t="shared" ref="AD2:AD18" si="3">(P2*Q2*Z2)^(1/3)</f>
+        <v>75.955590109188009</v>
       </c>
       <c r="AE2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="AF2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AH2">
+        <v>7</v>
+      </c>
+      <c r="AI2">
+        <f>AH2-4</f>
+        <v>3</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>116</v>
+      </c>
+      <c r="AK2">
+        <v>9</v>
+      </c>
+      <c r="AL2">
+        <f>AK2-6</f>
+        <v>3</v>
+      </c>
+      <c r="AM2">
+        <f t="shared" ref="AM2:AM18" si="4">G2-L2</f>
+        <v>5</v>
+      </c>
+      <c r="AN2" s="7">
+        <f t="shared" ref="AN2:AN18" si="5">(1-(45/J2))+0.2</f>
+        <v>0.63037974683544307</v>
+      </c>
+      <c r="AO2">
+        <f>0.65*J2</f>
+        <v>51.35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>7</v>
       </c>
@@ -1431,11 +1667,11 @@
         <v>73</v>
       </c>
       <c r="P3">
-        <f>(L3*N3*O3)^(1/3)</f>
+        <f t="shared" si="0"/>
         <v>72.655914952014115</v>
       </c>
       <c r="Q3">
-        <f>(F3*H3*K3)^(1/3)</f>
+        <f t="shared" si="1"/>
         <v>74.081235357026699</v>
       </c>
       <c r="R3" t="s">
@@ -1463,7 +1699,7 @@
         <v>0</v>
       </c>
       <c r="Z3">
-        <f>(T3*U3*V3*W3*X3)^(1/5)</f>
+        <f t="shared" si="2"/>
         <v>109.06474175824731</v>
       </c>
       <c r="AA3" s="2">
@@ -1476,7 +1712,7 @@
         <v>1</v>
       </c>
       <c r="AD3">
-        <f>(P3*Q3*Z3)^(1/3)</f>
+        <f t="shared" si="3"/>
         <v>83.731304197638465</v>
       </c>
       <c r="AE3" t="s">
@@ -1485,319 +1721,447 @@
       <c r="AF3" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG3" t="s">
+        <v>90</v>
+      </c>
+      <c r="AH3">
+        <v>8</v>
+      </c>
+      <c r="AI3">
+        <f>AH3-2</f>
+        <v>6</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>113</v>
+      </c>
+      <c r="AK3">
+        <v>7</v>
+      </c>
+      <c r="AL3">
+        <f>AK3-3</f>
+        <v>4</v>
+      </c>
+      <c r="AM3">
+        <f t="shared" si="4"/>
+        <v>4</v>
+      </c>
+      <c r="AN3" s="7">
+        <f t="shared" si="5"/>
+        <v>0.60789473684210527</v>
+      </c>
+      <c r="AO3">
+        <f t="shared" ref="AO3:AO18" si="6">0.65*J3</f>
+        <v>49.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4">
         <v>1000</v>
       </c>
       <c r="D4">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
+        <v>38</v>
+      </c>
+      <c r="G4">
+        <v>58</v>
+      </c>
+      <c r="H4">
         <v>61</v>
       </c>
-      <c r="G4">
+      <c r="I4">
+        <v>52</v>
+      </c>
+      <c r="J4">
+        <v>74</v>
+      </c>
+      <c r="K4">
+        <v>72</v>
+      </c>
+      <c r="L4">
+        <v>41</v>
+      </c>
+      <c r="M4">
+        <v>53</v>
+      </c>
+      <c r="N4">
+        <v>41</v>
+      </c>
+      <c r="O4">
+        <v>38</v>
+      </c>
+      <c r="P4">
+        <f t="shared" si="0"/>
+        <v>39.974567166034475</v>
+      </c>
+      <c r="Q4">
+        <f t="shared" si="1"/>
+        <v>55.057350645777831</v>
+      </c>
+      <c r="R4" t="s">
+        <v>43</v>
+      </c>
+      <c r="S4">
+        <v>30</v>
+      </c>
+      <c r="T4">
+        <v>83</v>
+      </c>
+      <c r="U4">
+        <v>96</v>
+      </c>
+      <c r="V4">
+        <v>88</v>
+      </c>
+      <c r="W4">
         <v>80</v>
       </c>
-      <c r="H4">
-        <v>80</v>
-      </c>
-      <c r="I4">
-        <v>75</v>
-      </c>
-      <c r="J4">
-        <v>63</v>
-      </c>
-      <c r="K4">
+      <c r="X4">
         <v>65</v>
-      </c>
-      <c r="L4">
-        <v>70</v>
-      </c>
-      <c r="M4">
-        <v>68</v>
-      </c>
-      <c r="N4">
-        <v>68</v>
-      </c>
-      <c r="O4">
-        <v>65</v>
-      </c>
-      <c r="P4">
-        <f>(L4*N4*O4)^(1/3)</f>
-        <v>67.635302453070338</v>
-      </c>
-      <c r="Q4">
-        <f>(F4*H4*K4)^(1/3)</f>
-        <v>68.19895596134819</v>
-      </c>
-      <c r="R4" t="s">
-        <v>42</v>
-      </c>
-      <c r="S4">
-        <v>22</v>
-      </c>
-      <c r="T4">
-        <v>91</v>
-      </c>
-      <c r="U4">
-        <v>101</v>
-      </c>
-      <c r="V4">
-        <v>104</v>
-      </c>
-      <c r="W4">
-        <v>88</v>
-      </c>
-      <c r="X4">
-        <v>106</v>
       </c>
       <c r="Y4">
         <v>0</v>
       </c>
       <c r="Z4">
-        <f>(T4*U4*V4*W4*X4)^(1/5)</f>
-        <v>97.732032010306668</v>
-      </c>
-      <c r="AA4">
-        <v>7</v>
-      </c>
-      <c r="AB4" s="2">
-        <v>3</v>
-      </c>
-      <c r="AC4" s="2">
-        <v>6</v>
+        <f t="shared" si="2"/>
+        <v>81.727284331662204</v>
+      </c>
+      <c r="AA4" s="1">
+        <v>15</v>
+      </c>
+      <c r="AB4">
+        <v>10</v>
+      </c>
+      <c r="AC4">
+        <v>10</v>
       </c>
       <c r="AD4">
-        <f>(P4*Q4*Z4)^(1/3)</f>
-        <v>76.676573510804658</v>
+        <f t="shared" si="3"/>
+        <v>56.448886890215348</v>
       </c>
       <c r="AE4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="AF4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>103</v>
+      </c>
+      <c r="AH4">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="AI4">
+        <f>AH4-13</f>
+        <v>-4.1999999999999993</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>125</v>
+      </c>
+      <c r="AK4">
+        <v>9</v>
+      </c>
+      <c r="AL4">
+        <f>AK4-15</f>
+        <v>-6</v>
+      </c>
+      <c r="AM4">
+        <f t="shared" si="4"/>
+        <v>17</v>
+      </c>
+      <c r="AN4" s="7">
+        <f t="shared" si="5"/>
+        <v>0.59189189189189184</v>
+      </c>
+      <c r="AO4">
+        <f t="shared" si="6"/>
+        <v>48.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C5">
         <v>1000</v>
       </c>
       <c r="D5">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>48</v>
-      </c>
-      <c r="G5">
-        <v>79</v>
+        <v>78</v>
+      </c>
+      <c r="G5" s="1">
+        <v>40</v>
       </c>
       <c r="H5">
+        <v>46</v>
+      </c>
+      <c r="I5">
         <v>80</v>
       </c>
-      <c r="I5">
-        <v>78</v>
-      </c>
       <c r="J5">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="K5">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L5">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="M5">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N5">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="O5">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="P5">
-        <f>(L5*N5*O5)^(1/3)</f>
-        <v>68.434216775695589</v>
+        <f t="shared" si="0"/>
+        <v>68.545213193224626</v>
       </c>
       <c r="Q5">
-        <f>(F5*H5*K5)^(1/3)</f>
-        <v>64.537145840981722</v>
+        <f t="shared" si="1"/>
+        <v>62.486631807533421</v>
       </c>
       <c r="R5" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="S5">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="T5">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="U5">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="V5">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="W5">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="X5">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="Y5">
         <v>0</v>
       </c>
       <c r="Z5">
-        <f>(T5*U5*V5*W5*X5)^(1/5)</f>
-        <v>99.219302709069495</v>
+        <f t="shared" si="2"/>
+        <v>101.40429546223</v>
       </c>
       <c r="AA5" s="2">
+        <v>5</v>
+      </c>
+      <c r="AB5" s="2">
         <v>6</v>
       </c>
-      <c r="AB5" s="2">
-        <v>4</v>
-      </c>
       <c r="AC5" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AD5">
-        <f>(P5*Q5*Z5)^(1/3)</f>
-        <v>75.955590109188009</v>
+        <f t="shared" si="3"/>
+        <v>75.730972363733088</v>
       </c>
       <c r="AE5" t="s">
         <v>65</v>
       </c>
       <c r="AF5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>94</v>
+      </c>
+      <c r="AH5">
+        <v>8.5709999999999997</v>
+      </c>
+      <c r="AI5">
+        <f>AH5-5</f>
+        <v>3.5709999999999997</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AK5">
+        <v>8.5709999999999997</v>
+      </c>
+      <c r="AL5">
+        <f>AK5-5</f>
+        <v>3.5709999999999997</v>
+      </c>
+      <c r="AM5">
+        <f t="shared" si="4"/>
+        <v>-32</v>
+      </c>
+      <c r="AN5" s="7">
+        <f t="shared" si="5"/>
+        <v>0.59189189189189184</v>
+      </c>
+      <c r="AO5">
+        <f t="shared" si="6"/>
+        <v>48.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C6">
         <v>1000</v>
       </c>
       <c r="D6">
-        <v>73</v>
+        <v>38</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
       <c r="F6">
-        <v>78</v>
-      </c>
-      <c r="G6">
-        <v>40</v>
+        <v>41</v>
+      </c>
+      <c r="G6" s="1">
+        <v>36</v>
       </c>
       <c r="H6">
+        <v>42</v>
+      </c>
+      <c r="I6">
+        <v>61</v>
+      </c>
+      <c r="J6">
+        <v>73</v>
+      </c>
+      <c r="K6">
+        <v>69</v>
+      </c>
+      <c r="L6">
+        <v>54</v>
+      </c>
+      <c r="M6">
+        <v>68</v>
+      </c>
+      <c r="N6">
+        <v>63</v>
+      </c>
+      <c r="O6">
+        <v>50</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="0"/>
+        <v>55.407442513434958</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="1"/>
+        <v>49.161758902384868</v>
+      </c>
+      <c r="R6" t="s">
+        <v>45</v>
+      </c>
+      <c r="S6">
+        <v>20</v>
+      </c>
+      <c r="T6">
+        <v>90</v>
+      </c>
+      <c r="U6">
+        <v>85</v>
+      </c>
+      <c r="V6">
         <v>46</v>
       </c>
-      <c r="I6">
-        <v>80</v>
-      </c>
-      <c r="J6">
-        <v>74</v>
-      </c>
-      <c r="K6">
-        <v>68</v>
-      </c>
-      <c r="L6">
-        <v>72</v>
-      </c>
-      <c r="M6">
-        <v>73</v>
-      </c>
-      <c r="N6">
-        <v>71</v>
-      </c>
-      <c r="O6">
-        <v>63</v>
-      </c>
-      <c r="P6">
-        <f>(L6*N6*O6)^(1/3)</f>
-        <v>68.545213193224626</v>
-      </c>
-      <c r="Q6">
-        <f>(F6*H6*K6)^(1/3)</f>
-        <v>62.486631807533421</v>
-      </c>
-      <c r="R6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S6">
-        <v>39</v>
-      </c>
-      <c r="T6">
-        <v>98</v>
-      </c>
-      <c r="U6">
-        <v>104</v>
-      </c>
-      <c r="V6">
-        <v>93</v>
-      </c>
       <c r="W6">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="X6">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="Y6">
         <v>0</v>
       </c>
       <c r="Z6">
-        <f>(T6*U6*V6*W6*X6)^(1/5)</f>
-        <v>101.40429546223</v>
-      </c>
-      <c r="AA6" s="2">
-        <v>5</v>
-      </c>
-      <c r="AB6" s="2">
-        <v>6</v>
-      </c>
-      <c r="AC6" s="2">
-        <v>3</v>
+        <f t="shared" si="2"/>
+        <v>80.475871292938109</v>
+      </c>
+      <c r="AA6">
+        <v>11</v>
+      </c>
+      <c r="AB6" s="1">
+        <v>13</v>
+      </c>
+      <c r="AC6">
+        <v>11</v>
       </c>
       <c r="AD6">
-        <f>(P6*Q6*Z6)^(1/3)</f>
-        <v>75.730972363733088</v>
+        <f t="shared" si="3"/>
+        <v>60.295800896964579</v>
       </c>
       <c r="AE6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="AF6" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>101</v>
+      </c>
+      <c r="AH6">
+        <v>10.75</v>
+      </c>
+      <c r="AI6">
+        <f>AH6-12</f>
+        <v>-1.25</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>121</v>
+      </c>
+      <c r="AK6">
+        <v>11</v>
+      </c>
+      <c r="AL6">
+        <f>AK6-11</f>
+        <v>0</v>
+      </c>
+      <c r="AM6">
+        <f t="shared" si="4"/>
+        <v>-18</v>
+      </c>
+      <c r="AN6" s="7">
+        <f t="shared" si="5"/>
+        <v>0.58356164383561637</v>
+      </c>
+      <c r="AO6">
+        <f t="shared" si="6"/>
+        <v>47.45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C7">
         <v>1000</v>
@@ -1809,709 +2173,1029 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G7">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="H7">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="I7">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="J7">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="K7">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="L7">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="M7">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="N7">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="O7">
-        <v>58</v>
+        <v>80</v>
       </c>
       <c r="P7">
-        <f>(L7*N7*O7)^(1/3)</f>
-        <v>65.119150290655128</v>
+        <f t="shared" si="0"/>
+        <v>78.661048467230643</v>
       </c>
       <c r="Q7">
-        <f>(F7*H7*K7)^(1/3)</f>
-        <v>63.933198527852717</v>
+        <f t="shared" si="1"/>
+        <v>69.38785980258659</v>
       </c>
       <c r="R7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="S7">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="T7">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="U7">
+        <v>115</v>
+      </c>
+      <c r="V7">
+        <v>111</v>
+      </c>
+      <c r="W7">
         <v>106</v>
       </c>
-      <c r="V7">
-        <v>86</v>
-      </c>
-      <c r="W7">
-        <v>101</v>
-      </c>
       <c r="X7">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="Y7">
         <v>0</v>
       </c>
       <c r="Z7">
-        <f>(T7*U7*V7*W7*X7)^(1/5)</f>
-        <v>93.535481974801968</v>
-      </c>
-      <c r="AA7">
-        <v>8</v>
+        <f t="shared" si="2"/>
+        <v>108.3103906739629</v>
+      </c>
+      <c r="AA7" s="2">
+        <v>1</v>
       </c>
       <c r="AB7" s="2">
-        <v>5</v>
-      </c>
-      <c r="AC7">
-        <v>7</v>
+        <v>2</v>
+      </c>
+      <c r="AC7" s="2">
+        <v>2</v>
       </c>
       <c r="AD7">
-        <f>(P7*Q7*Z7)^(1/3)</f>
-        <v>73.024823385404346</v>
+        <f t="shared" si="3"/>
+        <v>83.92753126291089</v>
       </c>
       <c r="AE7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="AF7" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>89</v>
+      </c>
+      <c r="AH7">
+        <v>8.3330000000000002</v>
+      </c>
+      <c r="AI7">
+        <f>AH7-1</f>
+        <v>7.3330000000000002</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>111</v>
+      </c>
+      <c r="AK7">
+        <v>6.3330000000000002</v>
+      </c>
+      <c r="AL7">
+        <f>AK7-1</f>
+        <v>5.3330000000000002</v>
+      </c>
+      <c r="AM7">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="AN7" s="7">
+        <f t="shared" si="5"/>
+        <v>0.56619718309859146</v>
+      </c>
+      <c r="AO7">
+        <f t="shared" si="6"/>
+        <v>46.15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C8">
         <v>1000</v>
       </c>
       <c r="D8">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="F8">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="G8">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="H8">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="I8">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="J8">
         <v>65</v>
       </c>
       <c r="K8">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L8">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="M8">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="N8">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="O8">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="P8">
-        <f>(L8*N8*O8)^(1/3)</f>
-        <v>73.313470286134418</v>
+        <f t="shared" si="0"/>
+        <v>65.119150290655128</v>
       </c>
       <c r="Q8">
-        <f>(F8*H8*K8)^(1/3)</f>
-        <v>52.761956065898168</v>
+        <f t="shared" si="1"/>
+        <v>63.933198527852717</v>
       </c>
       <c r="R8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="S8">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="T8">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="U8">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="V8">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="W8">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="X8">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="Y8">
         <v>0</v>
       </c>
       <c r="Z8">
-        <f>(T8*U8*V8*W8*X8)^(1/5)</f>
-        <v>99.292960339357776</v>
-      </c>
-      <c r="AA8" s="2">
-        <v>2</v>
-      </c>
-      <c r="AB8" s="1">
-        <v>12</v>
-      </c>
-      <c r="AC8" s="2">
-        <v>4</v>
+        <f t="shared" si="2"/>
+        <v>93.535481974801968</v>
+      </c>
+      <c r="AA8">
+        <v>8</v>
+      </c>
+      <c r="AB8" s="2">
+        <v>5</v>
+      </c>
+      <c r="AC8">
+        <v>7</v>
       </c>
       <c r="AD8">
-        <f>(P8*Q8*Z8)^(1/3)</f>
-        <v>72.689950774447908</v>
+        <f t="shared" si="3"/>
+        <v>73.024823385404346</v>
       </c>
       <c r="AE8" t="s">
         <v>66</v>
       </c>
       <c r="AF8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+      <c r="AG8" t="s">
+        <v>95</v>
+      </c>
+      <c r="AH8">
+        <v>13</v>
+      </c>
+      <c r="AI8">
+        <f>AH8-6</f>
+        <v>7</v>
+      </c>
+      <c r="AJ8" t="s">
+        <v>118</v>
+      </c>
+      <c r="AK8">
+        <v>14</v>
+      </c>
+      <c r="AL8">
+        <f>AK8-8</f>
+        <v>6</v>
+      </c>
+      <c r="AM8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AN8" s="7">
+        <f t="shared" si="5"/>
+        <v>0.50769230769230766</v>
+      </c>
+      <c r="AO8">
+        <f t="shared" si="6"/>
+        <v>42.25</v>
+      </c>
+      <c r="AP8" s="7">
+        <f>1-(AO8^2/2025)</f>
+        <v>0.11848765432098762</v>
+      </c>
+      <c r="AQ8">
+        <f>G8-(2/3*L8)</f>
+        <v>23</v>
+      </c>
+      <c r="AR8">
+        <f>2*((5*AQ8)/(SQRT(((H8+AO8)/2)+AQ8)))</f>
+        <v>26.448140430499173</v>
+      </c>
+      <c r="AS8">
+        <f>AO8+AR8</f>
+        <v>68.698140430499166</v>
+      </c>
+    </row>
+    <row r="9" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C9">
         <v>1000</v>
       </c>
       <c r="D9">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
       <c r="F9">
-        <v>53</v>
-      </c>
-      <c r="G9">
-        <v>69</v>
+        <v>51</v>
+      </c>
+      <c r="G9" s="1">
+        <v>52</v>
       </c>
       <c r="H9">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="I9">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="J9">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="K9">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="L9">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="M9">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="N9">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="O9">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="P9">
-        <f>(L9*N9*O9)^(1/3)</f>
-        <v>64.07673088570175</v>
+        <f t="shared" si="0"/>
+        <v>73.313470286134418</v>
       </c>
       <c r="Q9">
-        <f>(F9*H9*K9)^(1/3)</f>
-        <v>55.634201650752019</v>
+        <f t="shared" si="1"/>
+        <v>52.761956065898168</v>
       </c>
       <c r="R9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S9">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="T9">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="U9">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="V9">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="W9">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="X9">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="Y9">
         <v>0</v>
       </c>
       <c r="Z9">
-        <f>(T9*U9*V9*W9*X9)^(1/5)</f>
-        <v>88.849913225041462</v>
-      </c>
-      <c r="AA9">
-        <v>9</v>
-      </c>
-      <c r="AB9">
-        <v>9</v>
-      </c>
-      <c r="AC9">
-        <v>9</v>
+        <f t="shared" si="2"/>
+        <v>99.292960339357776</v>
+      </c>
+      <c r="AA9" s="2">
+        <v>2</v>
+      </c>
+      <c r="AB9" s="1">
+        <v>12</v>
+      </c>
+      <c r="AC9" s="2">
+        <v>4</v>
       </c>
       <c r="AD9">
-        <f>(P9*Q9*Z9)^(1/3)</f>
-        <v>68.165779428031499</v>
+        <f t="shared" si="3"/>
+        <v>72.689950774447908</v>
       </c>
       <c r="AE9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="AF9" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>96</v>
+      </c>
+      <c r="AH9">
+        <v>11.4</v>
+      </c>
+      <c r="AI9">
+        <f>AH9-7</f>
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="AJ9" t="s">
+        <v>112</v>
+      </c>
+      <c r="AK9">
+        <v>11.4</v>
+      </c>
+      <c r="AL9">
+        <f>AK9-2</f>
+        <v>9.4</v>
+      </c>
+      <c r="AM9">
+        <f t="shared" si="4"/>
+        <v>-22</v>
+      </c>
+      <c r="AN9" s="7">
+        <f t="shared" si="5"/>
+        <v>0.50769230769230766</v>
+      </c>
+      <c r="AO9">
+        <f t="shared" si="6"/>
+        <v>42.25</v>
+      </c>
+      <c r="AP9" s="7">
+        <f t="shared" ref="AP8:AP18" si="7">1-(AO9^2/2025)</f>
+        <v>0.11848765432098762</v>
+      </c>
+      <c r="AQ9">
+        <f t="shared" ref="AQ9:AQ18" si="8">G9-(2/3*L9)</f>
+        <v>2.6666666666666714</v>
+      </c>
+      <c r="AR9">
+        <f t="shared" ref="AR9:AR18" si="9">2*((5*AQ9)/(SQRT(((H9+AO9)/2)+AQ9)))</f>
+        <v>3.8573819521220436</v>
+      </c>
+      <c r="AS9">
+        <f t="shared" ref="AS9:AS18" si="10">AO9+AR9</f>
+        <v>46.10738195212204</v>
+      </c>
+    </row>
+    <row r="10" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C10">
         <v>1000</v>
       </c>
       <c r="D10">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
       <c r="F10">
-        <v>44</v>
-      </c>
-      <c r="G10">
-        <v>68</v>
+        <v>65</v>
+      </c>
+      <c r="G10" s="1">
+        <v>48</v>
       </c>
       <c r="H10">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="I10">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J10">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="K10">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="L10">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="M10">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="N10">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="O10">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="P10">
-        <f>(L10*N10*O10)^(1/3)</f>
-        <v>59.642691212493077</v>
+        <f t="shared" si="0"/>
+        <v>69.182879701160502</v>
       </c>
       <c r="Q10">
-        <f>(F10*H10*K10)^(1/3)</f>
-        <v>54.993938725981302</v>
+        <f t="shared" si="1"/>
+        <v>57.205170119664565</v>
       </c>
       <c r="R10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="S10">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="T10">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="U10">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="V10">
-        <v>105</v>
+        <v>31</v>
       </c>
       <c r="W10">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="X10">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="Y10">
         <v>0</v>
       </c>
       <c r="Z10">
-        <f>(T10*U10*V10*W10*X10)^(1/5)</f>
-        <v>91.78614003552201</v>
-      </c>
-      <c r="AA10">
-        <v>10</v>
+        <f t="shared" si="2"/>
+        <v>68.04457550548446</v>
+      </c>
+      <c r="AA10" s="2">
+        <v>4</v>
       </c>
       <c r="AB10">
-        <v>11</v>
-      </c>
-      <c r="AC10">
         <v>8</v>
       </c>
+      <c r="AC10" s="1">
+        <v>16</v>
+      </c>
       <c r="AD10">
-        <f>(P10*Q10*Z10)^(1/3)</f>
-        <v>67.021846351328719</v>
+        <f t="shared" si="3"/>
+        <v>64.576694157456615</v>
       </c>
       <c r="AE10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="AF10" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>99</v>
+      </c>
+      <c r="AH10">
+        <v>3.3330000000000002</v>
+      </c>
+      <c r="AI10">
+        <f>AH10-10</f>
+        <v>-6.6669999999999998</v>
+      </c>
+      <c r="AJ10" t="s">
+        <v>114</v>
+      </c>
+      <c r="AK10">
+        <v>5</v>
+      </c>
+      <c r="AL10">
+        <f>AK10-4</f>
+        <v>1</v>
+      </c>
+      <c r="AM10">
+        <f t="shared" si="4"/>
+        <v>-25</v>
+      </c>
+      <c r="AN10" s="7">
+        <f t="shared" si="5"/>
+        <v>0.50769230769230766</v>
+      </c>
+      <c r="AO10">
+        <f t="shared" si="6"/>
+        <v>42.25</v>
+      </c>
+      <c r="AP10" s="7">
+        <f t="shared" si="7"/>
+        <v>0.11848765432098762</v>
+      </c>
+      <c r="AQ10">
+        <f t="shared" si="8"/>
+        <v>-0.6666666666666643</v>
+      </c>
+      <c r="AR10">
+        <f t="shared" si="9"/>
+        <v>-1.0171500602514383</v>
+      </c>
+      <c r="AS10">
+        <f t="shared" si="10"/>
+        <v>41.232849939748561</v>
+      </c>
+    </row>
+    <row r="11" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C11">
         <v>1000</v>
       </c>
       <c r="D11">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11">
+        <v>61</v>
+      </c>
+      <c r="G11">
+        <v>80</v>
+      </c>
+      <c r="H11">
+        <v>80</v>
+      </c>
+      <c r="I11">
+        <v>75</v>
+      </c>
+      <c r="J11">
+        <v>63</v>
+      </c>
+      <c r="K11">
         <v>65</v>
       </c>
-      <c r="G11">
-        <v>48</v>
-      </c>
-      <c r="H11">
-        <v>45</v>
-      </c>
-      <c r="I11">
-        <v>73</v>
-      </c>
-      <c r="J11">
+      <c r="L11">
+        <v>70</v>
+      </c>
+      <c r="M11">
+        <v>68</v>
+      </c>
+      <c r="N11">
+        <v>68</v>
+      </c>
+      <c r="O11">
         <v>65</v>
       </c>
-      <c r="K11">
-        <v>64</v>
-      </c>
-      <c r="L11">
-        <v>73</v>
-      </c>
-      <c r="M11">
-        <v>61</v>
-      </c>
-      <c r="N11">
-        <v>72</v>
-      </c>
-      <c r="O11">
-        <v>63</v>
-      </c>
       <c r="P11">
-        <f>(L11*N11*O11)^(1/3)</f>
-        <v>69.182879701160502</v>
+        <f t="shared" si="0"/>
+        <v>67.635302453070338</v>
       </c>
       <c r="Q11">
-        <f>(F11*H11*K11)^(1/3)</f>
-        <v>57.205170119664565</v>
+        <f t="shared" si="1"/>
+        <v>68.19895596134819</v>
       </c>
       <c r="R11" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="S11">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="T11">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="U11">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="V11">
-        <v>31</v>
+        <v>104</v>
       </c>
       <c r="W11">
         <v>88</v>
       </c>
       <c r="X11">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="Y11">
         <v>0</v>
       </c>
       <c r="Z11">
-        <f>(T11*U11*V11*W11*X11)^(1/5)</f>
-        <v>68.04457550548446</v>
-      </c>
-      <c r="AA11" s="2">
+        <f t="shared" si="2"/>
+        <v>97.732032010306668</v>
+      </c>
+      <c r="AA11">
+        <v>7</v>
+      </c>
+      <c r="AB11" s="2">
+        <v>3</v>
+      </c>
+      <c r="AC11" s="2">
+        <v>6</v>
+      </c>
+      <c r="AD11">
+        <f t="shared" si="3"/>
+        <v>76.676573510804658</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG11" t="s">
+        <v>92</v>
+      </c>
+      <c r="AH11">
+        <v>6.3330000000000002</v>
+      </c>
+      <c r="AI11">
+        <f>AH11-3</f>
+        <v>3.3330000000000002</v>
+      </c>
+      <c r="AJ11" t="s">
+        <v>117</v>
+      </c>
+      <c r="AK11">
+        <v>5</v>
+      </c>
+      <c r="AL11">
+        <f>AK11-7</f>
+        <v>-2</v>
+      </c>
+      <c r="AM11">
+        <f t="shared" si="4"/>
+        <v>10</v>
+      </c>
+      <c r="AN11" s="7">
+        <f t="shared" si="5"/>
+        <v>0.48571428571428571</v>
+      </c>
+      <c r="AO11">
+        <f t="shared" si="6"/>
+        <v>40.950000000000003</v>
+      </c>
+      <c r="AP11" s="7">
+        <f t="shared" si="7"/>
+        <v>0.17189999999999994</v>
+      </c>
+      <c r="AQ11">
+        <f t="shared" si="8"/>
+        <v>33.333333333333336</v>
+      </c>
+      <c r="AR11">
+        <f t="shared" si="9"/>
+        <v>34.415813156121459</v>
+      </c>
+      <c r="AS11">
+        <f t="shared" si="10"/>
+        <v>75.365813156121462</v>
+      </c>
+    </row>
+    <row r="12" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>4</v>
       </c>
-      <c r="AB11">
-        <v>8</v>
-      </c>
-      <c r="AC11" s="1">
-        <v>16</v>
-      </c>
-      <c r="AD11">
-        <f>(P11*Q11*Z11)^(1/3)</f>
-        <v>64.576694157456615</v>
-      </c>
-      <c r="AE11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF11" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>13</v>
-      </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="C12">
         <v>1000</v>
       </c>
       <c r="D12">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
       <c r="F12">
+        <v>44</v>
+      </c>
+      <c r="G12">
         <v>68</v>
       </c>
-      <c r="G12">
-        <v>57</v>
-      </c>
       <c r="H12">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="I12">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="J12">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="K12">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="L12">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="M12">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="N12">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="O12">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="P12">
-        <f>(L12*N12*O12)^(1/3)</f>
-        <v>51.897232933730805</v>
+        <f t="shared" si="0"/>
+        <v>59.642691212493077</v>
       </c>
       <c r="Q12">
-        <f>(F12*H12*K12)^(1/3)</f>
-        <v>57.570348679045033</v>
+        <f t="shared" si="1"/>
+        <v>54.993938725981302</v>
       </c>
       <c r="R12" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="S12">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="T12">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="U12">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="V12">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="W12">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="X12">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="Y12">
         <v>0</v>
       </c>
       <c r="Z12">
-        <f>(T12*U12*V12*W12*X12)^(1/5)</f>
-        <v>76.519639730270072</v>
-      </c>
-      <c r="AA12" s="1">
-        <v>12</v>
+        <f t="shared" si="2"/>
+        <v>91.78614003552201</v>
+      </c>
+      <c r="AA12">
+        <v>10</v>
       </c>
       <c r="AB12">
-        <v>7</v>
-      </c>
-      <c r="AC12" s="1">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="AC12">
+        <v>8</v>
       </c>
       <c r="AD12">
-        <f>(P12*Q12*Z12)^(1/3)</f>
-        <v>61.146554878976481</v>
+        <f t="shared" si="3"/>
+        <v>67.021846351328719</v>
       </c>
       <c r="AE12" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="AF12" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="AG12" t="s">
+        <v>98</v>
+      </c>
+      <c r="AH12">
+        <v>12.25</v>
+      </c>
+      <c r="AI12">
+        <f>AH12-9</f>
+        <v>3.25</v>
+      </c>
+      <c r="AJ12" t="s">
+        <v>120</v>
+      </c>
+      <c r="AK12">
+        <v>12.25</v>
+      </c>
+      <c r="AL12">
+        <f>AK12-10</f>
+        <v>2.25</v>
+      </c>
+      <c r="AM12">
+        <f t="shared" si="4"/>
+        <v>6</v>
+      </c>
+      <c r="AN12" s="7">
+        <f t="shared" si="5"/>
+        <v>0.43728813559322038</v>
+      </c>
+      <c r="AO12">
+        <f t="shared" si="6"/>
+        <v>38.35</v>
+      </c>
+      <c r="AP12" s="7">
+        <f t="shared" si="7"/>
+        <v>0.27371728395061723</v>
+      </c>
+      <c r="AQ12">
+        <f t="shared" si="8"/>
+        <v>26.666666666666671</v>
+      </c>
+      <c r="AR12">
+        <f t="shared" si="9"/>
+        <v>29.658631154382181</v>
+      </c>
+      <c r="AS12">
+        <f t="shared" si="10"/>
+        <v>68.008631154382186</v>
+      </c>
+    </row>
+    <row r="13" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C13">
         <v>1000</v>
       </c>
       <c r="D13">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
       <c r="F13">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="G13">
-        <v>36</v>
+        <v>69</v>
       </c>
       <c r="H13">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="I13">
         <v>61</v>
       </c>
       <c r="J13">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="K13">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="L13">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="M13">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="N13">
+        <v>72</v>
+      </c>
+      <c r="O13">
         <v>63</v>
       </c>
-      <c r="O13">
+      <c r="P13">
+        <f t="shared" si="0"/>
+        <v>64.07673088570175</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="1"/>
+        <v>55.634201650752019</v>
+      </c>
+      <c r="R13" t="s">
         <v>50</v>
       </c>
-      <c r="P13">
-        <f>(L13*N13*O13)^(1/3)</f>
-        <v>55.407442513434958</v>
-      </c>
-      <c r="Q13">
-        <f>(F13*H13*K13)^(1/3)</f>
-        <v>49.161758902384868</v>
-      </c>
-      <c r="R13" t="s">
-        <v>45</v>
-      </c>
       <c r="S13">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="T13">
+        <v>86</v>
+      </c>
+      <c r="U13">
         <v>90</v>
       </c>
-      <c r="U13">
-        <v>85</v>
-      </c>
       <c r="V13">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="W13">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="X13">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="Y13">
         <v>0</v>
       </c>
       <c r="Z13">
-        <f>(T13*U13*V13*W13*X13)^(1/5)</f>
-        <v>80.475871292938109</v>
+        <f t="shared" si="2"/>
+        <v>88.849913225041462</v>
       </c>
       <c r="AA13">
+        <v>9</v>
+      </c>
+      <c r="AB13">
+        <v>9</v>
+      </c>
+      <c r="AC13">
+        <v>9</v>
+      </c>
+      <c r="AD13">
+        <f t="shared" si="3"/>
+        <v>68.165779428031499</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>64</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG13" t="s">
+        <v>97</v>
+      </c>
+      <c r="AH13">
+        <v>12</v>
+      </c>
+      <c r="AI13">
+        <f>AH13-8</f>
+        <v>4</v>
+      </c>
+      <c r="AJ13" t="s">
+        <v>119</v>
+      </c>
+      <c r="AK13">
         <v>11</v>
       </c>
-      <c r="AB13" s="1">
-        <v>13</v>
-      </c>
-      <c r="AC13">
+      <c r="AL13">
+        <f>AK13-9</f>
+        <v>2</v>
+      </c>
+      <c r="AM13">
+        <f t="shared" si="4"/>
         <v>11</v>
       </c>
-      <c r="AD13">
-        <f>(P13*Q13*Z13)^(1/3)</f>
-        <v>60.295800896964579</v>
-      </c>
-      <c r="AE13" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF13" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AN13" s="7">
+        <f t="shared" si="5"/>
+        <v>0.42413793103448277</v>
+      </c>
+      <c r="AO13">
+        <f t="shared" si="6"/>
+        <v>37.700000000000003</v>
+      </c>
+      <c r="AP13" s="7">
+        <f t="shared" si="7"/>
+        <v>0.29812839506172828</v>
+      </c>
+      <c r="AQ13">
+        <f t="shared" si="8"/>
+        <v>30.333333333333336</v>
+      </c>
+      <c r="AR13">
+        <f t="shared" si="9"/>
+        <v>34.415668618263226</v>
+      </c>
+      <c r="AS13">
+        <f t="shared" si="10"/>
+        <v>72.115668618263228</v>
+      </c>
+    </row>
+    <row r="14" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C14">
         <v>1000</v>
@@ -2523,296 +3207,440 @@
         <v>0</v>
       </c>
       <c r="F14">
+        <v>40</v>
+      </c>
+      <c r="G14">
         <v>38</v>
       </c>
-      <c r="G14">
-        <v>58</v>
-      </c>
       <c r="H14">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="I14">
+        <v>51</v>
+      </c>
+      <c r="J14">
+        <v>50</v>
+      </c>
+      <c r="K14">
+        <v>48</v>
+      </c>
+      <c r="L14">
+        <v>38</v>
+      </c>
+      <c r="M14">
+        <v>47</v>
+      </c>
+      <c r="N14">
+        <v>31</v>
+      </c>
+      <c r="O14">
+        <v>35</v>
+      </c>
+      <c r="P14">
+        <f t="shared" si="0"/>
+        <v>34.546531066931053</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" si="1"/>
+        <v>41.039422720240729</v>
+      </c>
+      <c r="R14" t="s">
+        <v>49</v>
+      </c>
+      <c r="S14">
+        <v>11</v>
+      </c>
+      <c r="T14">
+        <v>86</v>
+      </c>
+      <c r="U14">
         <v>52</v>
       </c>
-      <c r="J14">
-        <v>74</v>
-      </c>
-      <c r="K14">
-        <v>72</v>
-      </c>
-      <c r="L14">
-        <v>41</v>
-      </c>
-      <c r="M14">
-        <v>53</v>
-      </c>
-      <c r="N14">
-        <v>41</v>
-      </c>
-      <c r="O14">
-        <v>38</v>
-      </c>
-      <c r="P14">
-        <f>(L14*N14*O14)^(1/3)</f>
-        <v>39.974567166034475</v>
-      </c>
-      <c r="Q14">
-        <f>(F14*H14*K14)^(1/3)</f>
-        <v>55.057350645777831</v>
-      </c>
-      <c r="R14" t="s">
-        <v>43</v>
-      </c>
-      <c r="S14">
-        <v>30</v>
-      </c>
-      <c r="T14">
-        <v>83</v>
-      </c>
-      <c r="U14">
-        <v>96</v>
-      </c>
       <c r="V14">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="W14">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="X14">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="Y14">
         <v>0</v>
       </c>
       <c r="Z14">
-        <f>(T14*U14*V14*W14*X14)^(1/5)</f>
-        <v>81.727284331662204</v>
+        <f t="shared" si="2"/>
+        <v>70.608359130094755</v>
       </c>
       <c r="AA14" s="1">
+        <v>16</v>
+      </c>
+      <c r="AB14" s="1">
+        <v>14</v>
+      </c>
+      <c r="AC14" s="1">
         <v>15</v>
       </c>
-      <c r="AB14">
-        <v>10</v>
-      </c>
-      <c r="AC14">
-        <v>10</v>
-      </c>
       <c r="AD14">
-        <f>(P14*Q14*Z14)^(1/3)</f>
-        <v>56.448886890215348</v>
+        <f t="shared" si="3"/>
+        <v>46.432343366746572</v>
       </c>
       <c r="AE14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="AF14" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+      <c r="AG14" t="s">
+        <v>104</v>
+      </c>
+      <c r="AH14">
+        <v>10.25</v>
+      </c>
+      <c r="AI14">
+        <f>AH14-15</f>
+        <v>-4.75</v>
+      </c>
+      <c r="AJ14" t="s">
+        <v>126</v>
+      </c>
+      <c r="AK14">
+        <v>9.75</v>
+      </c>
+      <c r="AL14">
+        <f>AK14-16</f>
+        <v>-6.25</v>
+      </c>
+      <c r="AM14">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AN14" s="7">
+        <f t="shared" si="5"/>
+        <v>0.3</v>
+      </c>
+      <c r="AO14">
+        <f t="shared" si="6"/>
+        <v>32.5</v>
+      </c>
+      <c r="AP14" s="7">
+        <f t="shared" si="7"/>
+        <v>0.47839506172839508</v>
+      </c>
+      <c r="AQ14">
+        <f t="shared" si="8"/>
+        <v>12.666666666666668</v>
+      </c>
+      <c r="AR14">
+        <f t="shared" si="9"/>
+        <v>18.492633708592344</v>
+      </c>
+      <c r="AS14">
+        <f t="shared" si="10"/>
+        <v>50.992633708592344</v>
+      </c>
+    </row>
+    <row r="15" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="D15">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E15">
         <v>0</v>
       </c>
       <c r="F15">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G15">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="H15">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I15">
+        <v>42</v>
+      </c>
+      <c r="J15">
+        <v>46</v>
+      </c>
+      <c r="K15">
+        <v>45</v>
+      </c>
+      <c r="L15">
+        <v>21</v>
+      </c>
+      <c r="M15">
+        <v>45</v>
+      </c>
+      <c r="N15">
         <v>26</v>
       </c>
-      <c r="J15">
-        <v>24</v>
-      </c>
-      <c r="K15">
-        <v>38</v>
-      </c>
-      <c r="L15">
-        <v>48</v>
-      </c>
-      <c r="M15">
-        <v>23</v>
-      </c>
-      <c r="N15">
-        <v>53</v>
-      </c>
       <c r="O15">
+        <v>27</v>
+      </c>
+      <c r="P15">
+        <f t="shared" si="0"/>
+        <v>24.519906076689331</v>
+      </c>
+      <c r="Q15">
+        <f t="shared" si="1"/>
+        <v>32.991733466587988</v>
+      </c>
+      <c r="R15" t="s">
         <v>51</v>
       </c>
-      <c r="P15">
-        <f>(L15*N15*O15)^(1/3)</f>
-        <v>50.624695928672054</v>
-      </c>
-      <c r="Q15">
-        <f>(F15*H15*K15)^(1/3)</f>
-        <v>30.545573721448037</v>
-      </c>
-      <c r="R15" t="s">
-        <v>40</v>
-      </c>
       <c r="S15">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="T15">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="U15">
+        <v>36</v>
+      </c>
+      <c r="V15">
+        <v>52</v>
+      </c>
+      <c r="W15">
+        <v>60</v>
+      </c>
+      <c r="X15">
         <v>81</v>
-      </c>
-      <c r="V15">
-        <v>83</v>
-      </c>
-      <c r="W15">
-        <v>46</v>
-      </c>
-      <c r="X15">
-        <v>70</v>
       </c>
       <c r="Y15">
         <v>0</v>
       </c>
       <c r="Z15">
-        <f>(T15*U15*V15*W15*X15)^(1/5)</f>
-        <v>72.883382116408441</v>
+        <f t="shared" si="2"/>
+        <v>60.622930273266903</v>
       </c>
       <c r="AA15" s="1">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AB15" s="1">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AC15" s="1">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AD15">
-        <f>(P15*Q15*Z15)^(1/3)</f>
-        <v>48.30362721438221</v>
+        <f t="shared" si="3"/>
+        <v>36.60330387601212</v>
       </c>
       <c r="AE15" t="s">
         <v>68</v>
       </c>
-      <c r="AF15" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AF15" t="s">
+        <v>79</v>
+      </c>
+      <c r="AG15" t="s">
+        <v>106</v>
+      </c>
+      <c r="AH15">
+        <v>10.25</v>
+      </c>
+      <c r="AI15">
+        <f>AH15-17</f>
+        <v>-6.75</v>
+      </c>
+      <c r="AJ15" t="s">
+        <v>127</v>
+      </c>
+      <c r="AK15">
+        <v>9.75</v>
+      </c>
+      <c r="AL15">
+        <f>AK15-17</f>
+        <v>-7.25</v>
+      </c>
+      <c r="AM15">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="AN15" s="7">
+        <f t="shared" si="5"/>
+        <v>0.22173913043478261</v>
+      </c>
+      <c r="AO15">
+        <f t="shared" si="6"/>
+        <v>29.900000000000002</v>
+      </c>
+      <c r="AP15" s="7">
+        <f t="shared" si="7"/>
+        <v>0.55851358024691355</v>
+      </c>
+      <c r="AQ15">
+        <f t="shared" si="8"/>
+        <v>10</v>
+      </c>
+      <c r="AR15">
+        <f t="shared" si="9"/>
+        <v>16.795459121697256</v>
+      </c>
+      <c r="AS15">
+        <f t="shared" si="10"/>
+        <v>46.695459121697255</v>
+      </c>
+    </row>
+    <row r="16" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C16">
         <v>1000</v>
       </c>
       <c r="D16">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="E16">
         <v>0</v>
       </c>
       <c r="F16">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="G16">
+        <v>57</v>
+      </c>
+      <c r="H16">
+        <v>61</v>
+      </c>
+      <c r="I16">
+        <v>48</v>
+      </c>
+      <c r="J16" s="1">
         <v>38</v>
       </c>
-      <c r="H16">
+      <c r="K16">
+        <v>46</v>
+      </c>
+      <c r="L16">
+        <v>52</v>
+      </c>
+      <c r="M16">
         <v>36</v>
       </c>
-      <c r="I16">
-        <v>51</v>
-      </c>
-      <c r="J16">
-        <v>50</v>
-      </c>
-      <c r="K16">
+      <c r="N16">
+        <v>56</v>
+      </c>
+      <c r="O16">
         <v>48</v>
       </c>
-      <c r="L16">
-        <v>38</v>
-      </c>
-      <c r="M16">
-        <v>47</v>
-      </c>
-      <c r="N16">
-        <v>31</v>
-      </c>
-      <c r="O16">
-        <v>35</v>
-      </c>
       <c r="P16">
-        <f>(L16*N16*O16)^(1/3)</f>
-        <v>34.546531066931053</v>
+        <f t="shared" si="0"/>
+        <v>51.897232933730805</v>
       </c>
       <c r="Q16">
-        <f>(F16*H16*K16)^(1/3)</f>
-        <v>41.039422720240729</v>
+        <f t="shared" si="1"/>
+        <v>57.570348679045033</v>
       </c>
       <c r="R16" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="S16">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="T16">
+        <v>73</v>
+      </c>
+      <c r="U16">
+        <v>98</v>
+      </c>
+      <c r="V16">
+        <v>82</v>
+      </c>
+      <c r="W16">
+        <v>52</v>
+      </c>
+      <c r="X16">
         <v>86</v>
-      </c>
-      <c r="U16">
-        <v>52</v>
-      </c>
-      <c r="V16">
-        <v>95</v>
-      </c>
-      <c r="W16">
-        <v>51</v>
-      </c>
-      <c r="X16">
-        <v>81</v>
       </c>
       <c r="Y16">
         <v>0</v>
       </c>
       <c r="Z16">
-        <f>(T16*U16*V16*W16*X16)^(1/5)</f>
-        <v>70.608359130094755</v>
+        <f t="shared" si="2"/>
+        <v>76.519639730270072</v>
       </c>
       <c r="AA16" s="1">
-        <v>16</v>
-      </c>
-      <c r="AB16" s="1">
-        <v>14</v>
+        <v>12</v>
+      </c>
+      <c r="AB16">
+        <v>7</v>
       </c>
       <c r="AC16" s="1">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="AD16">
-        <f>(P16*Q16*Z16)^(1/3)</f>
-        <v>46.432343366746572</v>
+        <f t="shared" si="3"/>
+        <v>61.146554878976481</v>
       </c>
       <c r="AE16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AF16" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+      <c r="AG16" t="s">
+        <v>100</v>
+      </c>
+      <c r="AH16">
+        <v>11.5</v>
+      </c>
+      <c r="AI16">
+        <f>AH16-11</f>
+        <v>0.5</v>
+      </c>
+      <c r="AJ16" t="s">
+        <v>122</v>
+      </c>
+      <c r="AK16">
+        <v>12.5</v>
+      </c>
+      <c r="AL16">
+        <f>AK16-12</f>
+        <v>0.5</v>
+      </c>
+      <c r="AM16">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="AN16" s="7">
+        <f t="shared" si="5"/>
+        <v>1.5789473684210631E-2</v>
+      </c>
+      <c r="AO16">
+        <f t="shared" si="6"/>
+        <v>24.7</v>
+      </c>
+      <c r="AP16" s="7">
+        <f t="shared" si="7"/>
+        <v>0.698720987654321</v>
+      </c>
+      <c r="AQ16">
+        <f t="shared" si="8"/>
+        <v>22.333333333333336</v>
+      </c>
+      <c r="AR16">
+        <f t="shared" si="9"/>
+        <v>27.662107529254303</v>
+      </c>
+      <c r="AS16">
+        <f t="shared" si="10"/>
+        <v>52.362107529254303</v>
+      </c>
+    </row>
+    <row r="17" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>8</v>
       </c>
@@ -2831,7 +3659,7 @@
       <c r="F17">
         <v>31</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="1">
         <v>25</v>
       </c>
       <c r="H17">
@@ -2840,7 +3668,7 @@
       <c r="I17">
         <v>21</v>
       </c>
-      <c r="J17">
+      <c r="J17" s="1">
         <v>31</v>
       </c>
       <c r="K17">
@@ -2859,11 +3687,11 @@
         <v>45</v>
       </c>
       <c r="P17">
-        <f>(L17*N17*O17)^(1/3)</f>
+        <f t="shared" si="0"/>
         <v>43.458938660650439</v>
       </c>
       <c r="Q17">
-        <f>(F17*H17*K17)^(1/3)</f>
+        <f t="shared" si="1"/>
         <v>26.728882509474577</v>
       </c>
       <c r="R17" t="s">
@@ -2891,7 +3719,7 @@
         <v>0</v>
       </c>
       <c r="Z17">
-        <f>(T17*U17*V17*W17*X17)^(1/5)</f>
+        <f t="shared" si="2"/>
         <v>72.190306479738268</v>
       </c>
       <c r="AA17" s="1">
@@ -2904,7 +3732,7 @@
         <v>14</v>
       </c>
       <c r="AD17">
-        <f>(P17*Q17*Z17)^(1/3)</f>
+        <f t="shared" si="3"/>
         <v>43.770307852044496</v>
       </c>
       <c r="AE17" t="s">
@@ -2913,112 +3741,585 @@
       <c r="AF17" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG17" t="s">
+        <v>105</v>
+      </c>
+      <c r="AH17">
+        <v>6.2859999999999996</v>
+      </c>
+      <c r="AI17">
+        <f>AH17-16</f>
+        <v>-9.7140000000000004</v>
+      </c>
+      <c r="AJ17" t="s">
+        <v>124</v>
+      </c>
+      <c r="AK17">
+        <v>5.8570000000000002</v>
+      </c>
+      <c r="AL17">
+        <f>AK17-14</f>
+        <v>-8.1430000000000007</v>
+      </c>
+      <c r="AM17">
+        <f t="shared" si="4"/>
+        <v>-13</v>
+      </c>
+      <c r="AN17" s="7">
+        <f t="shared" si="5"/>
+        <v>-0.25161290322580648</v>
+      </c>
+      <c r="AO17">
+        <f t="shared" si="6"/>
+        <v>20.150000000000002</v>
+      </c>
+      <c r="AP17" s="7">
+        <f t="shared" si="7"/>
+        <v>0.79949506172839502</v>
+      </c>
+      <c r="AQ17">
+        <f t="shared" si="8"/>
+        <v>-0.33333333333333215</v>
+      </c>
+      <c r="AR17">
+        <f t="shared" si="9"/>
+        <v>-0.68410559711236441</v>
+      </c>
+      <c r="AS17">
+        <f t="shared" si="10"/>
+        <v>19.465894402887638</v>
+      </c>
+    </row>
+    <row r="18" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C18">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E18">
         <v>0</v>
       </c>
       <c r="F18">
+        <v>25</v>
+      </c>
+      <c r="G18" s="1">
+        <v>44</v>
+      </c>
+      <c r="H18">
+        <v>30</v>
+      </c>
+      <c r="I18">
+        <v>26</v>
+      </c>
+      <c r="J18" s="1">
+        <v>24</v>
+      </c>
+      <c r="K18">
         <v>38</v>
       </c>
-      <c r="G18">
-        <v>24</v>
-      </c>
-      <c r="H18">
+      <c r="L18">
+        <v>48</v>
+      </c>
+      <c r="M18">
+        <v>23</v>
+      </c>
+      <c r="N18">
+        <v>53</v>
+      </c>
+      <c r="O18">
+        <v>51</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="0"/>
+        <v>50.624695928672054</v>
+      </c>
+      <c r="Q18">
+        <f t="shared" si="1"/>
+        <v>30.545573721448037</v>
+      </c>
+      <c r="R18" t="s">
+        <v>40</v>
+      </c>
+      <c r="S18">
         <v>21</v>
       </c>
-      <c r="I18">
-        <v>42</v>
-      </c>
-      <c r="J18">
+      <c r="T18">
+        <v>95</v>
+      </c>
+      <c r="U18">
+        <v>81</v>
+      </c>
+      <c r="V18">
+        <v>83</v>
+      </c>
+      <c r="W18">
         <v>46</v>
       </c>
-      <c r="K18">
-        <v>45</v>
-      </c>
-      <c r="L18">
-        <v>21</v>
-      </c>
-      <c r="M18">
-        <v>45</v>
-      </c>
-      <c r="N18">
-        <v>26</v>
-      </c>
-      <c r="O18">
-        <v>27</v>
-      </c>
-      <c r="P18">
-        <f>(L18*N18*O18)^(1/3)</f>
-        <v>24.519906076689331</v>
-      </c>
-      <c r="Q18">
-        <f>(F18*H18*K18)^(1/3)</f>
-        <v>32.991733466587988</v>
-      </c>
-      <c r="R18" t="s">
-        <v>51</v>
-      </c>
-      <c r="S18">
-        <v>39</v>
-      </c>
-      <c r="T18">
-        <v>90</v>
-      </c>
-      <c r="U18">
-        <v>36</v>
-      </c>
-      <c r="V18">
-        <v>52</v>
-      </c>
-      <c r="W18">
-        <v>60</v>
-      </c>
       <c r="X18">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="Y18">
         <v>0</v>
       </c>
       <c r="Z18">
-        <f>(T18*U18*V18*W18*X18)^(1/5)</f>
-        <v>60.622930273266903</v>
+        <f t="shared" si="2"/>
+        <v>72.883382116408441</v>
       </c>
       <c r="AA18" s="1">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="AB18" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AC18" s="1">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="AD18">
-        <f>(P18*Q18*Z18)^(1/3)</f>
-        <v>36.60330387601212</v>
+        <f t="shared" si="3"/>
+        <v>48.30362721438221</v>
       </c>
       <c r="AE18" t="s">
         <v>68</v>
       </c>
-      <c r="AF18" t="s">
+      <c r="AF18" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AG18" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="AH18">
+        <v>13</v>
+      </c>
+      <c r="AI18">
+        <f>AH18-14</f>
+        <v>-1</v>
+      </c>
+      <c r="AJ18" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="AK18">
+        <v>15</v>
+      </c>
+      <c r="AL18">
+        <f>AK18-13</f>
+        <v>2</v>
+      </c>
+      <c r="AM18">
+        <f t="shared" si="4"/>
+        <v>-4</v>
+      </c>
+      <c r="AN18" s="7">
+        <f t="shared" si="5"/>
+        <v>-0.67500000000000004</v>
+      </c>
+      <c r="AO18">
+        <f t="shared" si="6"/>
+        <v>15.600000000000001</v>
+      </c>
+      <c r="AP18" s="7">
+        <f t="shared" si="7"/>
+        <v>0.87982222222222217</v>
+      </c>
+      <c r="AQ18">
+        <f t="shared" si="8"/>
+        <v>12</v>
+      </c>
+      <c r="AR18">
+        <f t="shared" si="9"/>
+        <v>20.341905108624314</v>
+      </c>
+      <c r="AS18">
+        <f t="shared" si="10"/>
+        <v>35.941905108624312</v>
+      </c>
+    </row>
+    <row r="20" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AA20" s="2"/>
+      <c r="AB20" s="2"/>
+      <c r="AC20" s="2"/>
+    </row>
+    <row r="21" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AA21" s="2"/>
+      <c r="AB21" s="2"/>
+      <c r="AC21" s="2"/>
+    </row>
+    <row r="23" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AB23" s="1"/>
+    </row>
+    <row r="24" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AA24" s="1"/>
+      <c r="AB24" s="1"/>
+      <c r="AC24" s="1"/>
+      <c r="AF24" s="3"/>
+      <c r="AG24" s="6"/>
+      <c r="AJ24" s="6"/>
+    </row>
+    <row r="26" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AB26" s="1"/>
+    </row>
+    <row r="27" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AB27" s="1"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AN18" xr:uid="{94A9DEAF-4754-41E1-A6D8-10B03E1EEF36}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AN18">
+      <sortCondition descending="1" ref="AN1:AN18"/>
+    </sortState>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A20:B24">
+    <sortCondition ref="A20:A24"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AC47F2C-966E-47B9-B41E-DD5DB5B4AC46}">
+  <dimension ref="A2:B18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
         <v>79</v>
       </c>
     </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" t="s">
+        <v>85</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AF18">
-    <sortCondition descending="1" ref="AD2:AD18"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D62FBA0-BF08-445E-BCCD-AFF8EB7E60BD}">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="4">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="4">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>38</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="5">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11">
+        <v>48</v>
+      </c>
+      <c r="D11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>51</v>
+      </c>
+      <c r="D12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13">
+        <v>53</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="5">
+        <v>74</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D2:E13">
+    <sortCondition ref="E2:E13"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>